<commit_message>
Implement hybrid offline-first saving and fix bugs
</commit_message>
<xml_diff>
--- a/registros_diarios/registros_ingreso_2025-07-01.xlsx
+++ b/registros_diarios/registros_ingreso_2025-07-01.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="68">
   <si>
     <t>DNI</t>
   </si>
@@ -212,9 +212,6 @@
   </si>
   <si>
     <t>Allcover</t>
-  </si>
-  <si>
-    <t>N/A</t>
   </si>
   <si>
     <t>ROJO</t>
@@ -227,16 +224,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -252,7 +241,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -260,30 +249,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -582,28 +553,28 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -615,7 +586,7 @@
         <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -626,7 +597,7 @@
         <v>22</v>
       </c>
       <c r="H3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -649,7 +620,7 @@
         <v>63</v>
       </c>
       <c r="H4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -660,7 +631,7 @@
         <v>24</v>
       </c>
       <c r="H5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -671,7 +642,7 @@
         <v>25</v>
       </c>
       <c r="H6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -694,7 +665,7 @@
         <v>63</v>
       </c>
       <c r="H7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -708,7 +679,7 @@
         <v>27</v>
       </c>
       <c r="H8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -722,7 +693,7 @@
         <v>28</v>
       </c>
       <c r="H9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -736,7 +707,7 @@
         <v>29</v>
       </c>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -750,7 +721,7 @@
         <v>30</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -764,7 +735,7 @@
         <v>31</v>
       </c>
       <c r="H12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -778,7 +749,7 @@
         <v>32</v>
       </c>
       <c r="H13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -792,7 +763,7 @@
         <v>33</v>
       </c>
       <c r="H14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -806,7 +777,7 @@
         <v>34</v>
       </c>
       <c r="H15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -820,7 +791,7 @@
         <v>35</v>
       </c>
       <c r="H16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -834,7 +805,7 @@
         <v>36</v>
       </c>
       <c r="H17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -848,7 +819,7 @@
         <v>37</v>
       </c>
       <c r="H18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -862,7 +833,7 @@
         <v>38</v>
       </c>
       <c r="H19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -885,7 +856,7 @@
         <v>64</v>
       </c>
       <c r="H20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -908,7 +879,7 @@
         <v>65</v>
       </c>
       <c r="H21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -919,7 +890,7 @@
         <v>41</v>
       </c>
       <c r="H22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -942,7 +913,7 @@
         <v>63</v>
       </c>
       <c r="H23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -956,7 +927,7 @@
         <v>43</v>
       </c>
       <c r="H24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -979,7 +950,7 @@
         <v>64</v>
       </c>
       <c r="H25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -993,7 +964,7 @@
         <v>45</v>
       </c>
       <c r="H26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1016,7 +987,7 @@
         <v>64</v>
       </c>
       <c r="H27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1039,7 +1010,7 @@
         <v>65</v>
       </c>
       <c r="H28" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1053,7 +1024,7 @@
         <v>48</v>
       </c>
       <c r="H29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1076,7 +1047,7 @@
         <v>63</v>
       </c>
       <c r="H30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1090,7 +1061,7 @@
         <v>50</v>
       </c>
       <c r="H31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -1113,7 +1084,7 @@
         <v>64</v>
       </c>
       <c r="H32" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -1136,7 +1107,7 @@
         <v>64</v>
       </c>
       <c r="H33" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -1159,7 +1130,7 @@
         <v>64</v>
       </c>
       <c r="H34" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -1182,7 +1153,7 @@
         <v>63</v>
       </c>
       <c r="H35" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -1205,7 +1176,7 @@
         <v>65</v>
       </c>
       <c r="H36" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -1228,7 +1199,7 @@
         <v>64</v>
       </c>
       <c r="H37" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -1251,7 +1222,7 @@
         <v>65</v>
       </c>
       <c r="H38" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -1273,11 +1244,8 @@
       <c r="F39" t="s">
         <v>63</v>
       </c>
-      <c r="G39" t="s">
-        <v>66</v>
-      </c>
       <c r="H39" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>